<commit_message>
Scenario Optimizer created with dynamic grouping included
</commit_message>
<xml_diff>
--- a/tests/data/test_scenarios/test_1/separate/test_bid_file1.xlsx
+++ b/tests/data/test_scenarios/test_1/separate/test_bid_file1.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PHWATES\OneDrive - kochind.com\Documents\Ad hoc\RFP Analysis Automation Files\OneDrive_2024-09-16\RFP Submissions\RFP data test\Dummy data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chrisw78\RFP Automation REPO\RFP_Analysis_Automation2\tests\data\test_scenarios\test_1\separate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFD8E0BD-F147-4231-BF56-BD070CF62166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F594D38-9246-4C49-A1F1-13BF2BB1E11C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3225" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1A7BC2FC-647D-4157-9E99-863769B2D979}"/>
+    <workbookView xWindow="-28920" yWindow="1890" windowWidth="29040" windowHeight="15720" xr2:uid="{1A7BC2FC-647D-4157-9E99-863769B2D979}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="rebates" sheetId="2" r:id="rId2"/>
+    <sheet name="capacity" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
   <si>
     <t>Bid ID</t>
   </si>
@@ -56,9 +58,6 @@
     <t>Facility</t>
   </si>
   <si>
-    <t>Supplier 1</t>
-  </si>
-  <si>
     <t>Facility 1</t>
   </si>
   <si>
@@ -72,19 +71,68 @@
   </si>
   <si>
     <t>Facility 5</t>
+  </si>
+  <si>
+    <t>Supplier Name</t>
+  </si>
+  <si>
+    <t>Min Volume</t>
+  </si>
+  <si>
+    <t>Max Volume</t>
+  </si>
+  <si>
+    <t>Min Spend</t>
+  </si>
+  <si>
+    <t>Max Spend</t>
+  </si>
+  <si>
+    <t>% Rebate</t>
+  </si>
+  <si>
+    <t>$ Rebate</t>
+  </si>
+  <si>
+    <t>Grouping</t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t>Chris</t>
+  </si>
+  <si>
+    <t>Cationic</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -110,9 +158,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,7 +542,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C2">
         <v>3437457</v>
@@ -494,7 +554,7 @@
         <v>0.05</v>
       </c>
       <c r="F2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -502,7 +562,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C3">
         <v>3001110</v>
@@ -514,7 +574,7 @@
         <v>1.1982124563104641</v>
       </c>
       <c r="F3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -522,7 +582,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C4">
         <v>24000</v>
@@ -534,7 +594,7 @@
         <v>0.80197197492137406</v>
       </c>
       <c r="F4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -542,7 +602,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C5">
         <v>357800</v>
@@ -554,7 +614,7 @@
         <v>1.4546193605527693</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -562,7 +622,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C6">
         <v>45000</v>
@@ -574,7 +634,7 @@
         <v>0.36439431543408707</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -585,7 +645,180 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04C18635-EF8D-47D2-B7D3-A593DBFDC414}">
+  <dimension ref="A1:N23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2001</v>
+      </c>
+      <c r="C2" s="3">
+        <v>10000000000</v>
+      </c>
+      <c r="D2" s="3">
+        <v>4000</v>
+      </c>
+      <c r="E2" s="3">
+        <v>5000</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0.99</v>
+      </c>
+      <c r="G2" s="5">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="21" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+    </row>
+    <row r="22" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="5"/>
+    </row>
+    <row r="23" spans="8:14" x14ac:dyDescent="0.25">
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="GUID" r:id="rId1"/>
+  </customProperties>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B93E7737-A174-4399-97CE-07E7D9495EF2}">
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="7">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="21" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+    </row>
+    <row r="22" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="7"/>
+    </row>
+    <row r="23" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="GUID" r:id="rId1"/>
+  </customProperties>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_activity xmlns="36c84e8f-8e8b-4f16-afe9-157f6eb5b1e8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100775005CFD392BB4A8128C579084B7368" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d0ab1e07bd207cdfebf07432cd898d0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="36c84e8f-8e8b-4f16-afe9-157f6eb5b1e8" xmlns:ns4="0a7a5492-aa41-4e4f-84c5-5c4d2fc7ef62" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2203819e5208aac76c01b66f26f7dcb5" ns1:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -855,26 +1088,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947A5C1-63CF-4600-9A9A-353C59D44DE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="36c84e8f-8e8b-4f16-afe9-157f6eb5b1e8"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="0a7a5492-aa41-4e4f-84c5-5c4d2fc7ef62"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_activity xmlns="36c84e8f-8e8b-4f16-afe9-157f6eb5b1e8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4C2A12E-7701-4847-9DA9-C29FCAF6ACBC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B6A8B56-0B12-49F4-957B-8466EFE44B71}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -892,30 +1132,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4C2A12E-7701-4847-9DA9-C29FCAF6ACBC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947A5C1-63CF-4600-9A9A-353C59D44DE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="36c84e8f-8e8b-4f16-afe9-157f6eb5b1e8"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="0a7a5492-aa41-4e4f-84c5-5c4d2fc7ef62"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>